<commit_message>
Descriptive Statics Exersie 1
</commit_message>
<xml_diff>
--- a/week-01/Lab Work/DescriptiveStatics_EX1.xlsx
+++ b/week-01/Lab Work/DescriptiveStatics_EX1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Yu_Class 7\MOD 1\Class Lessons\Week 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nilla\Documents\Data-Analytics\week-01\Lab Work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D85EC39-4148-4D83-87DE-64884FFA31E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26594E50-A370-48DA-8D51-7FD0F9820541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2970" yWindow="1815" windowWidth="27870" windowHeight="12960" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sales_Data" sheetId="1" r:id="rId1"/>
@@ -219,9 +219,6 @@
     <t>3. What might management infer about customer satisfaction?</t>
   </si>
   <si>
-    <t xml:space="preserve">Management can infer that customers are very satisfied by the office supplies that they are buying. They can also infer that the customers feel a bit mediocore about the electronics that they are buying since the satisfaction is on the lower side of 4 stars and the start of 3 stars. Last but not least, for furnature management can infer that customers are feeling a bit unsatisfied with that product. Even though we only have a sample set of 5 for electronics and furnature, the data shows a negitive </t>
-  </si>
-  <si>
     <t>Part 3: Interpretation</t>
   </si>
   <si>
@@ -232,6 +229,9 @@
   </si>
   <si>
     <t>Some key insights that I discovered from the statistics is what products could be improved upon to increase customer satisfaction. Which regions are doing well, so management can see if their results can be duplicated to the other reigions. Using the data tab and having multipule custom sort filters helped me figure out what details management can infer about the customer satisfaction. I also learned how descriptive statistics highlights the different patterns that effect performance and highlight them for management.</t>
+  </si>
+  <si>
+    <t>Management can infer that customers are very satisfied by the office supplies that they are buying. They can also infer that the customers feel a bit mediocore about the electronics that they are buying since the satisfaction is on the lower side of 4 stars and the start of 3 stars. Last but not least, for furnature management can infer that customers are feeling a bit unsatisfied with that product. Even though we only have a sample set of 5 for electronics and furnature, the data shows a negitive corallation.</t>
   </si>
 </sst>
 </file>
@@ -241,7 +241,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -294,7 +294,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -305,6 +305,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 3" xfId="1" builtinId="18"/>
@@ -609,7 +613,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.140625" bestFit="1" customWidth="1"/>
@@ -620,7 +624,7 @@
     <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1" thickBot="1">
+    <row r="1" spans="1:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -646,7 +650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1001</v>
       </c>
@@ -672,7 +676,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1008</v>
       </c>
@@ -698,7 +702,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1020</v>
       </c>
@@ -724,7 +728,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>1013</v>
       </c>
@@ -750,7 +754,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>1015</v>
       </c>
@@ -776,7 +780,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>1003</v>
       </c>
@@ -802,7 +806,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>1006</v>
       </c>
@@ -828,7 +832,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>1018</v>
       </c>
@@ -854,7 +858,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>1011</v>
       </c>
@@ -880,7 +884,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>1002</v>
       </c>
@@ -906,7 +910,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>1005</v>
       </c>
@@ -932,7 +936,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>1010</v>
       </c>
@@ -958,7 +962,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>1016</v>
       </c>
@@ -984,7 +988,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>1012</v>
       </c>
@@ -1010,7 +1014,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>1009</v>
       </c>
@@ -1036,7 +1040,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>1017</v>
       </c>
@@ -1062,7 +1066,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>1004</v>
       </c>
@@ -1088,7 +1092,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>1007</v>
       </c>
@@ -1114,7 +1118,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>1014</v>
       </c>
@@ -1140,7 +1144,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>1019</v>
       </c>
@@ -1166,7 +1170,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="G22">
         <f>MEDIAN(G2:G21)</f>
         <v>1220</v>
@@ -1183,60 +1187,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:P50"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:P59"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" customWidth="1"/>
     <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="115.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="16" width="9.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1245,7 +1250,7 @@
         <v>1275.45</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1254,7 +1259,7 @@
         <v>1220</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1263,7 +1268,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1273,7 +1278,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="17" spans="1:15">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1282,7 +1287,7 @@
         <v>2370</v>
       </c>
     </row>
-    <row r="18" spans="1:15">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -1291,22 +1296,22 @@
         <v>742.04932982567732</v>
       </c>
     </row>
-    <row r="20" spans="1:15">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:15">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:15">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:15">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1335,7 +1340,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="25" spans="1:15">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1343,25 +1348,25 @@
         <v>39</v>
       </c>
     </row>
-    <row r="26" spans="1:15">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>40</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:15">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:15">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:15">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>44</v>
       </c>
@@ -1384,7 +1389,7 @@
         <v>490.29</v>
       </c>
     </row>
-    <row r="31" spans="1:15">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>45</v>
       </c>
@@ -1392,7 +1397,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:15">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -1400,17 +1405,17 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>49</v>
       </c>
@@ -1439,7 +1444,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>50</v>
       </c>
@@ -1447,7 +1452,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>51</v>
       </c>
@@ -1455,17 +1460,17 @@
         <v>52</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>55</v>
       </c>
@@ -1474,7 +1479,7 @@
         <v>4.3149999999999995</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>56</v>
       </c>
@@ -1493,35 +1498,121 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>59</v>
       </c>
-      <c r="H44" t="s">
+      <c r="H44" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="H45" s="7"/>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="46" spans="1:16">
-      <c r="A46" t="s">
+      <c r="H46" s="7"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="47" spans="1:16">
-      <c r="A47" t="s">
+      <c r="H47" s="7"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:16">
-      <c r="A48" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="7" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="50" spans="1:1">
-      <c r="A50" t="s">
-        <v>64</v>
-      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="7"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="7"/>
+      <c r="C55" s="7"/>
+      <c r="D55" s="7"/>
+      <c r="E55" s="7"/>
+      <c r="F55" s="7"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="7"/>
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
+      <c r="B58" s="7"/>
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="H44:H47"/>
+    <mergeCell ref="A50:F59"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>